<commit_message>
階段1: writer --trades-only 模式 + .writer.lock 互斥
--trades-only（Boss PC 第一段用）
  只寫 trades_all，不碰 CS交易紀錄／offset_state —— Boss 上根本沒有 CS 檔。
  gate() 的安全閘門一條未放寬（open/close 餘額明確性、needs_review、
  BALANCE 對不上／留倉／非交易現金）；冪等改查 trades_all 的 Date 欄。
  writer 被 gate 擋下時改回 exit 2，讓呼叫端腳本能靠 errorlevel 判斷。

回歸（11 案例，PASS）：4 案與生產檔逐格相同；5 案僅損益欄 str→float
（既有 writer 既有行為，已用完整 writer A/B 對照證明兩者輸出相同）；
2 案 gate 正確擋下（07-31 DOI 非交易現金、08-03 收盤留倉）。

.writer.lock
  常駐 app 會回寫整張 trades_all，而 openpyxl save 非原子操作，兩者相撞
  會互相蓋掉且無人看管下不會被發現。writer 寫入期間持鎖，app 見鎖即跳過
  回寫；鎖逾時 600 秒視為殘留，避免 writer 被中斷後 app 永遠停止回寫。

另附 setup_scheduled_task.ps1：兩台通用的 pythonw 開機常駐排程註冊腳本
（需系統管理員權限）。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trades_all.xlsx
+++ b/trades_all.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1381"/>
+  <dimension ref="A1:K1399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66643,6 +66643,852 @@
         </is>
       </c>
     </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>10:12:56</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1382" t="n">
+        <v>769.855</v>
+      </c>
+      <c r="G1382" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1382" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I1382" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1382" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1382" t="inlineStr">
+        <is>
+          <t>10:16:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>10:16:52</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1383" t="n">
+        <v>770.6701</v>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>多</t>
+        </is>
+      </c>
+      <c r="F1383" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="G1383" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1383" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I1383" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1383" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1383" t="inlineStr">
+        <is>
+          <t>10:12:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>10:25:04</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1384" t="n">
+        <v>772.2299</v>
+      </c>
+      <c r="G1384" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1384" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I1384" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1384" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1384" t="inlineStr">
+        <is>
+          <t>10:27:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>10:27:20</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1385" t="n">
+        <v>772.655</v>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>多</t>
+        </is>
+      </c>
+      <c r="F1385" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="G1385" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1385" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I1385" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1385" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1385" t="inlineStr">
+        <is>
+          <t>10:25:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>10:30:28</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1386" t="n">
+        <v>772.965</v>
+      </c>
+      <c r="G1386" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1386" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I1386" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1386" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1386" t="inlineStr">
+        <is>
+          <t>10:56:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>10:33:36</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1387" t="n">
+        <v>772.6108</v>
+      </c>
+      <c r="G1387" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1387" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I1387" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1387" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1387" t="inlineStr">
+        <is>
+          <t>10:56:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>10:56:10</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1388" t="n">
+        <v>772.6193</v>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>多</t>
+        </is>
+      </c>
+      <c r="F1388" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="G1388" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1388" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I1388" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1388" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1388" t="inlineStr">
+        <is>
+          <t>10:33:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>10:56:57</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1389" t="n">
+        <v>772.425</v>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>多</t>
+        </is>
+      </c>
+      <c r="F1389" t="n">
+        <v>-55.61</v>
+      </c>
+      <c r="G1389" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1389" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I1389" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1389" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1389" t="inlineStr">
+        <is>
+          <t>10:30:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>11:21:41</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1390" t="n">
+        <v>772.8996</v>
+      </c>
+      <c r="G1390" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1390" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I1390" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1390" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1390" t="inlineStr">
+        <is>
+          <t>11:23:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>11:23:34</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1391" t="n">
+        <v>773.4472</v>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>多</t>
+        </is>
+      </c>
+      <c r="F1391" t="n">
+        <v>53.15</v>
+      </c>
+      <c r="G1391" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1391" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I1391" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1391" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1391" t="inlineStr">
+        <is>
+          <t>11:21:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>11:36:55</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1392" t="n">
+        <v>773.4299</v>
+      </c>
+      <c r="G1392" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1392" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I1392" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1392" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1392" t="inlineStr">
+        <is>
+          <t>11:38:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>11:38:56</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1393" t="n">
+        <v>773.45</v>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>多</t>
+        </is>
+      </c>
+      <c r="F1393" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G1393" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1393" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I1393" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1393" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1393" t="inlineStr">
+        <is>
+          <t>11:36:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>11:41:18</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1394" t="n">
+        <v>773.4099</v>
+      </c>
+      <c r="G1394" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1394" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I1394" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1394" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1394" t="inlineStr">
+        <is>
+          <t>13:47:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>12:04:43</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1395" t="n">
+        <v>772.9645</v>
+      </c>
+      <c r="G1395" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1395" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I1395" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1395" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1395" t="inlineStr">
+        <is>
+          <t>12:07:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>12:07:01</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1396" t="n">
+        <v>773.3</v>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>多</t>
+        </is>
+      </c>
+      <c r="F1396" t="n">
+        <v>31.94</v>
+      </c>
+      <c r="G1396" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1396" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I1396" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1396" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1396" t="inlineStr">
+        <is>
+          <t>12:04:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>13:05:37</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1397" t="n">
+        <v>772.175</v>
+      </c>
+      <c r="G1397" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1397" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I1397" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1397" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1397" t="inlineStr">
+        <is>
+          <t>13:45:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>13:45:44</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1398" t="n">
+        <v>772.2313</v>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>多</t>
+        </is>
+      </c>
+      <c r="F1398" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="G1398" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1398" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I1398" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1398" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1398" t="inlineStr">
+        <is>
+          <t>13:05:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>13:47:32</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D1399" t="n">
+        <v>772.3749</v>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>多</t>
+        </is>
+      </c>
+      <c r="F1399" t="n">
+        <v>-105.11</v>
+      </c>
+      <c r="G1399" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1399" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I1399" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J1399" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K1399" t="inlineStr">
+        <is>
+          <t>11:41:18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>